<commit_message>
TEST-E201 : vérification indépendante appliquée — 5 détecteurs de fumée (A04) au lieu de 4 avertisseurs + 1, 6 recentrages
Agent vérificateur à l'aveugle (plan par zones + légende + rendu, sans CSV) : 0 écart de quantité, 0 omission,
0 faux positif ; famille M07 contestée → tranchée sur la légende E-001 au zoom x20 (A03 = 3/4 noir, A04 = diagonale) :
les 5 cercles sont A04. Décalages I05-01, I05-02, BJ, DM, int (i)/(j) corrigés par lecture ×12/×14. R-004 réécrite,
R-012 ajoutée, RAPPORT-VERIFICATEUR.md versionné. 19 familles, 121 repères, conforme=True.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TPwM3NeUDtfRgDUM5aSU7Z
</commit_message>
<xml_diff>
--- a/dossiers/TEST-E201/releve.xlsx
+++ b/dossiers/TEST-E201/releve.xlsx
@@ -478,7 +478,7 @@
         <v>121</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -653,20 +653,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AVERTISSEUR FUMEE 120V CO</t>
+          <t>BOITE JONCTION</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>alarme</t>
+          <t>distribution</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cercle 3/4 noir (R-004).</t>
+          <t>Carre X en tete de rail.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -678,20 +678,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOITE JONCTION</t>
+          <t>BOITIER C</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>distribution</t>
+          <t>autre</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Carre X en tete de rail.</t>
+          <t>C dans carre, hors legende.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -703,20 +703,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOITIER C</t>
+          <t>CERCLE SANS ETIQUETTE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>autre</t>
+          <t>luminaire</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C dans carre, hors legende.</t>
+          <t>Cercle simple ~8 pt sans etiquette ni circuit (R-005).</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -728,20 +728,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CERCLE SANS ETIQUETTE</t>
+          <t>DETECTEUR FUMEE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luminaire</t>
+          <t>alarme</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cercle simple ~8 pt sans etiquette ni circuit (R-005).</t>
+          <t>Cercle coupe en diagonale, moitie noire (A04). 5 au plan ; aucun avertisseur 3/4 noir (A03) — tranche au zoom x20 sur legende et plan (R-004).</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -753,20 +753,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DETECTEUR FUMEE</t>
+          <t>DETECTEUR MOUVEMENT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>alarme</t>
+          <t>commande</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cercle 1/2 noir (R-004).</t>
+          <t>Ovale DM.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -778,20 +778,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DETECTEUR MOUVEMENT</t>
+          <t>ENCASTRE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>commande</t>
+          <t>luminaire</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ovale DM.</t>
+          <t>Cercle + croix. Variante pleine = PP-U1 (urgence) : en designation.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -803,20 +803,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ENCASTRE</t>
+          <t>ENSEIGNE SORTIE MUR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>luminaire</t>
+          <t>secours</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cercle + croix. Variante pleine = PP-U1 (urgence) : en designation.</t>
+          <t>Cercle X mi-noir sur tige.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -828,7 +828,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ENSEIGNE SORTIE MUR</t>
+          <t>ENSEIGNE SORTIE PLAFOND</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -837,11 +837,11 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cercle X mi-noir sur tige.</t>
+          <t>Cercle X mi-noir avec fleche, sans tige.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -853,12 +853,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ENSEIGNE SORTIE PLAFOND</t>
+          <t>HP ENCASTRE PLAFOND</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>secours</t>
+          <t>alarme</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -866,7 +866,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Cercle X mi-noir avec fleche, sans tige.</t>
+          <t>Cercle avec carre.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -878,20 +878,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HP ENCASTRE PLAFOND</t>
+          <t>INT 3 VOIES</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>alarme</t>
+          <t>commande</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cercle avec carre.</t>
+          <t>$ avec 3 ; lettre de zone en designation.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -903,7 +903,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INT 3 VOIES</t>
+          <t>INT MAITRES</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>$ avec 3 ; lettre de zone en designation.</t>
+          <t>$ dans un carre + bulle 1 ; note specifique 1 : a relocaliser.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>INT MAITRES</t>
+          <t>INT SIMPLE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -937,11 +937,11 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>$ dans un carre + bulle 1 ; note specifique 1 : a relocaliser.</t>
+          <t>$ seul.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -953,20 +953,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INT SIMPLE</t>
+          <t>LED 1X4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>commande</t>
+          <t>luminaire</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>$ seul.</t>
+          <t>Rectangle a diagonale ; variante mi-noire = PP-U1 (urgence) en designation.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -978,7 +978,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LED 1X4</t>
+          <t>LED 2X2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -987,11 +987,11 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Rectangle a diagonale ; variante mi-noire = PP-U1 (urgence) en designation.</t>
+          <t>Carre a diagonale. Variante mi-noire = alimente par PP-U1 (urgence) : en designation.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1003,20 +1003,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LED 2X2</t>
+          <t>PANNEAU ANNONCIATEUR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>luminaire</t>
+          <t>alarme</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Carre a diagonale. Variante mi-noire = alimente par PP-U1 (urgence) : en designation.</t>
+          <t>ANN dans carre ; E.A.R.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1028,7 +1028,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PANNEAU ANNONCIATEUR</t>
+          <t>PIEZO STROBE</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1037,11 +1037,11 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ANN dans carre ; E.A.R.</t>
+          <t>F dans carre avec rayons.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1053,12 +1053,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PIEZO STROBE</t>
+          <t>RAIL ECLAIRAGE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>alarme</t>
+          <t>luminaire</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>F dans carre avec rayons.</t>
+          <t>Rail courbe avec tetes orientables ; 1 repere par rail, nb de tetes en designation (R-008).</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1078,48 +1078,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RAIL ECLAIRAGE</t>
+          <t>STATION MANUELLE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>luminaire</t>
+          <t>alarme</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Rail courbe avec tetes orientables ; 1 repere par rail, nb de tetes en designation (R-008).</t>
+          <t>F dans carre.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
-        <is>
-          <t>E-001 legende ; E-201 plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>STATION MANUELLE</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>alarme</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>3</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>F dans carre.</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
         <is>
           <t>E-001 legende ; E-201 plan</t>
         </is>
@@ -1136,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1200,11 +1175,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AVERTISSEUR FUMEE 120V CO</t>
+          <t>BOITE JONCTION</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1220,11 +1195,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BOITE JONCTION</t>
+          <t>BOITIER C</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1240,11 +1215,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BOITIER C</t>
+          <t>CERCLE SANS ETIQUETTE</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1260,11 +1235,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CERCLE SANS ETIQUETTE</t>
+          <t>DETECTEUR FUMEE</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1280,11 +1255,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DETECTEUR FUMEE</t>
+          <t>DETECTEUR MOUVEMENT</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1300,11 +1275,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DETECTEUR MOUVEMENT</t>
+          <t>ENCASTRE</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -1320,11 +1295,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ENCASTRE</t>
+          <t>ENSEIGNE SORTIE MUR</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1340,11 +1315,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ENSEIGNE SORTIE MUR</t>
+          <t>ENSEIGNE SORTIE PLAFOND</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1360,7 +1335,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ENSEIGNE SORTIE PLAFOND</t>
+          <t>HP ENCASTRE PLAFOND</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1380,11 +1355,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>HP ENCASTRE PLAFOND</t>
+          <t>INT 3 VOIES</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1400,11 +1375,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>INT 3 VOIES</t>
+          <t>INT MAITRES</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1420,11 +1395,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>INT MAITRES</t>
+          <t>INT SIMPLE</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1440,11 +1415,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>INT SIMPLE</t>
+          <t>LED 1X4</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -1460,11 +1435,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LED 1X4</t>
+          <t>LED 2X2</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17">
@@ -1480,11 +1455,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LED 2X2</t>
+          <t>PANNEAU ANNONCIATEUR</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1500,11 +1475,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PANNEAU ANNONCIATEUR</t>
+          <t>PIEZO STROBE</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1520,7 +1495,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PIEZO STROBE</t>
+          <t>RAIL ECLAIRAGE</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1540,30 +1515,10 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>RAIL ECLAIRAGE</t>
+          <t>STATION MANUELLE</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>E201</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>E201plan-p01</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>STATION MANUELLE</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3088,12 +3043,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>843.6</t>
+          <t>843.4</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>638.5</t>
+          <t>638.3</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3125,12 +3080,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>798.8</t>
+          <t>798.6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>658.6</t>
+          <t>658.4</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3162,12 +3117,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>860.8</t>
+          <t>860.6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>676.2</t>
+          <t>676.0</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3199,12 +3154,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>754.5</t>
+          <t>754.2</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>679.1</t>
+          <t>678.9</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3236,12 +3191,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>816.0</t>
+          <t>815.8</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>696.7</t>
+          <t>696.5</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3273,12 +3228,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>771.6</t>
+          <t>771.4</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>716.8</t>
+          <t>716.6</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3421,12 +3376,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>995.2</t>
+          <t>995.0</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>466.4</t>
+          <t>466.6</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3495,12 +3450,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1022.4</t>
+          <t>1022.2</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>526.3</t>
+          <t>526.1</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3569,12 +3524,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>1021.6</t>
+          <t>1021.4</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>557.3</t>
+          <t>557.0</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3606,12 +3561,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>976.8</t>
+          <t>977.0</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>577.8</t>
+          <t>577.6</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3643,12 +3598,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1038.7</t>
+          <t>1038.5</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>595.4</t>
+          <t>595.1</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3680,12 +3635,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>932.4</t>
+          <t>932.2</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>597.9</t>
+          <t>597.7</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3717,12 +3672,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>993.9</t>
+          <t>994.1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>615.5</t>
+          <t>615.2</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3754,12 +3709,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>949.6</t>
+          <t>949.8</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>636.0</t>
+          <t>635.3</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3791,12 +3746,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>1009.8</t>
+          <t>1009.6</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>740.6</t>
+          <t>740.4</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3828,12 +3783,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>932.4</t>
+          <t>932.6</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>818.9</t>
+          <t>819.1</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3865,12 +3820,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1094.8</t>
+          <t>1095.0</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>361.3</t>
+          <t>361.1</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3902,12 +3857,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>1151.4</t>
+          <t>1151.1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>363.8</t>
+          <t>364.0</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3939,12 +3894,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>1189.9</t>
+          <t>1189.7</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>365.1</t>
+          <t>364.9</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3976,12 +3931,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1189.9</t>
+          <t>1189.7</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>405.7</t>
+          <t>405.5</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4013,12 +3968,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>1094.8</t>
+          <t>1095.0</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>415.3</t>
+          <t>415.5</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4050,12 +4005,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>1189.9</t>
+          <t>1189.7</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>450.9</t>
+          <t>450.7</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -4087,12 +4042,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>1148.8</t>
+          <t>1148.6</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>493.6</t>
+          <t>493.4</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -4124,12 +4079,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>1078.9</t>
+          <t>1078.7</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>493.6</t>
+          <t>493.4</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -4161,12 +4116,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>1148.8</t>
+          <t>1148.6</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>544.7</t>
+          <t>544.5</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4198,12 +4153,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>1147.6</t>
+          <t>1147.4</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>602.1</t>
+          <t>601.8</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4235,12 +4190,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>1078.1</t>
+          <t>1078.3</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>672.0</t>
+          <t>671.8</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -4272,12 +4227,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>1078.9</t>
+          <t>1078.7</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>740.6</t>
+          <t>740.4</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4346,12 +4301,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>1029.5</t>
+          <t>1028.1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>348.5</t>
+          <t>345.6</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4383,12 +4338,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>977.6</t>
+          <t>980.3</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>412.0</t>
+          <t>410.5</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4420,7 +4375,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>1123.5</t>
+          <t>1121.0</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4457,12 +4412,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>331.5</t>
+          <t>331.4</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>907.8</t>
+          <t>907.5</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4494,12 +4449,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>565.2</t>
+          <t>566.7</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>811.0</t>
+          <t>813.7</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4531,12 +4486,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1203.7</t>
+          <t>1203.5</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>378.4</t>
+          <t>378.3</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4568,7 +4523,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>824.4</t>
+          <t>825.4</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4600,17 +4555,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AVERTISSEUR FUMEE 120V CO</t>
+          <t>DETECTEUR FUMEE</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>1033.5</t>
+          <t>1033.1</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>389.3</t>
+          <t>388.7</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4620,7 +4575,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>mesure raster : 86-92 % noir -&gt; 3/4 (L03 legende) ; voir R-004</t>
+          <t>symbole coupe en diagonale, moitie noire = A04 legende ; verifie au zoom x20 (verificateur independant + comparaison legende)</t>
         </is>
       </c>
     </row>
@@ -4637,17 +4592,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AVERTISSEUR FUMEE 120V CO</t>
+          <t>DETECTEUR FUMEE</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>541.2</t>
+          <t>540.7</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>377.4</t>
+          <t>377.0</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4657,7 +4612,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>mesure raster : 86-92 % noir -&gt; 3/4 (L03 legende) ; voir R-004</t>
+          <t>symbole coupe en diagonale, moitie noire = A04 legende ; verifie au zoom x20 (verificateur independant + comparaison legende)</t>
         </is>
       </c>
     </row>
@@ -4674,17 +4629,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AVERTISSEUR FUMEE 120V CO</t>
+          <t>DETECTEUR FUMEE</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>462.5</t>
+          <t>462.0</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>413.2</t>
+          <t>412.6</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4694,7 +4649,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>mesure raster : 86-92 % noir -&gt; 3/4 (L03 legende) ; voir R-004</t>
+          <t>symbole coupe en diagonale, moitie noire = A04 legende ; verifie au zoom x20 (verificateur independant + comparaison legende)</t>
         </is>
       </c>
     </row>
@@ -4711,17 +4666,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AVERTISSEUR FUMEE 120V CO</t>
+          <t>DETECTEUR FUMEE</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>881.9</t>
+          <t>880.7</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>704.4</t>
+          <t>704.8</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4731,7 +4686,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>E.A.R lu au zoom 780-950/600-730 ; voir R-004</t>
+          <t>symbole coupe en diagonale, moitie noire = A04 legende ; verifie au zoom x20 (verificateur independant + comparaison legende)</t>
         </is>
       </c>
     </row>
@@ -4827,12 +4782,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>1000.7</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>387.4</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4864,12 +4819,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1013</t>
+          <t>1011.6</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>420.5</t>
+          <t>417.4</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4901,12 +4856,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>1018.5</t>
+          <t>1016.9</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>414.5</t>
+          <t>415.9</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -5045,12 +5000,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>1076</t>
+          <t>1076.2</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>318</t>
+          <t>317.6</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -5082,12 +5037,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>519</t>
+          <t>518.9</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>853.5</t>
+          <t>851.4</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -5119,12 +5074,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>592</t>
+          <t>591.8</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>807</t>
+          <t>805.3</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5152,12 +5107,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>999.7</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>350.2</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -5189,12 +5144,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>1171</t>
+          <t>1170.8</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>340.3</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5300,12 +5255,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>431.5</t>
+          <t>431.4</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>850</t>
+          <t>849.9</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -5337,12 +5292,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>1143</t>
+          <t>1143.0</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>334.3</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5448,12 +5403,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>582</t>
+          <t>585.4</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>816</t>
+          <t>809.7</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5559,12 +5514,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>832</t>
+          <t>831.7</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>662</t>
+          <t>661.7</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5601,7 +5556,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>752</t>
+          <t>752.2</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5633,12 +5588,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>904.8</t>
+          <t>905.0</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>656</t>
+          <t>655.9</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5670,12 +5625,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>1083</t>
+          <t>1082.9</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>575</t>
+          <t>574.6</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5707,12 +5662,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>942.7</t>
+          <t>942.0</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>709.1</t>
+          <t>709.2</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5744,12 +5699,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>875.1</t>
+          <t>875.7</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>776.6</t>
+          <t>775.8</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5781,7 +5736,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>782.9</t>
+          <t>783.4</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5818,12 +5773,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>981.3</t>
+          <t>979.0</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>679.4</t>
+          <t>675.8</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5855,12 +5810,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>913.0</t>
+          <t>910.3</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>744.7</t>
+          <t>741.0</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5892,12 +5847,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>833.5</t>
+          <t>831.2</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>822.1</t>
+          <t>818.6</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -6003,12 +5958,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1154</t>
+          <t>1161.3</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>623</t>
+          <t>623.6</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -6040,12 +5995,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>1037</t>
+          <t>1038.5</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>785</t>
+          <t>790.0</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -6077,12 +6032,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>476</t>
+          <t>468.7</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>606.0</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -6237,7 +6192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -6379,257 +6334,313 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>## R-004 — Avertisseur 120 V CO (3/4 noir) vs détecteur de fumée (1/2 noir)</t>
+          <t>## R-004 — Détecteurs de fumée : les 5 petits cercles sont la ligne A04, pas A03</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Les 5 petits cercles (4,6 pt) ont été mesurés sur le raster : 86-92 % noir pour 4 d'entre eux → ligne A03</t>
+          <t>Première lecture : 4 « avertisseurs 120 V CO » (A03, 3/4 noir) + 1 « détecteur de fumée » (A04, 1/2 noir), d'après le</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>« avertisseur de fumée à ionisation 120 V combiné CO » ; 63 % pour celui de l'ascenseur (1146 ; 513) → A04</t>
+          <t>pourcentage de noir mesuré sur le raster. **Corrigé** après vérification indépendante : au zoom ×20, les 5 symboles</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>« détecteur de fumée ». La lecture repose sur la proportion de noir d'un symbole de 4,6 pt : **à confirmer** par</t>
+          <t>sont identiques — cercle coupé en diagonale, moitié noire — et la légende E-001 montre A03 = 3/4 noir (quart blanc en</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>l'estimateur sur le plan vectoriel. L'avertisseur (882 ; 704) porte E.A.R → RELOCALISER.</t>
+          <t>haut à gauche), A04 = coupé en diagonale. La mesure de noir était polluée par le trait de mur qui traverse 4 des 5</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>## R-005 — Deux cercles simples sans étiquette (905 ; 656) et (1083 ; 575)</t>
+          <t>symboles. Résultat : 5 × DÉTECTEUR DE FUMÉE (I01), dont 1 E.A.R (882 ; 704) ; aucun avertisseur 120 V sur E-201.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cercles noirs ~8 pt dans le corridor, sans PP ni circuit ni E.A.E. La légende L04 « appareil d'éclairage encastré »</t>
+          <t>Leçon : à 4,6 pt, une proportion de noir ne distingue pas deux lignes de légende ; comparer la forme au zoom.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>est un cercle simple, mais tous les autres encastrés de la feuille portent une croix et une étiquette. Relevés sous</t>
+          <t>## R-005 — Deux cercles simples sans étiquette (905 ; 656) et (1083 ; 575)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>« CERCLE SANS ETIQUETTE », portée `A PRECISER`. À trancher : luminaire ou symbole architectural.</t>
+          <t>Cercles noirs ~8 pt dans le corridor, sans PP ni circuit ni E.A.E. La légende L04 « appareil d'éclairage encastré »</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>## R-006 — Boîtier « C » (4 occurrences) hors légende</t>
+          <t>est un cercle simple, mais tous les autres encastrés de la feuille portent une croix et une étiquette. Relevés sous</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Carré portant « C », toujours près d'une porte (1143 ; 334), (1109 ; 367), (1017 ; 542), (582 ; 816 — E.A.E).</t>
+          <t>« CERCLE SANS ETIQUETTE », portée `A PRECISER`. À trancher : luminaire ou symbole architectural.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Absent des légendes E-001 (ni ÉLECTRICITÉ, ni ALARME INCENDIE/INTRUSION, ni SERVICES). Relevé sous « BOITIER C »,</t>
+          <t>## R-006 — Boîtier « C » (4 occurrences) hors légende</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>famille `autre`, matériel suffixé (hors legende). À identifier (contact de porte ? bouton de sortie ?).</t>
+          <t>Carré portant « C », toujours près d'une porte (1143 ; 334), (1109 ; 367), (1017 ; 542), (582 ; 816 — E.A.E).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>## R-007 — Interrupteurs maîtres (note spécifique 1)</t>
+          <t>Absent des légendes E-001 (ni ÉLECTRICITÉ, ni ALARME INCENDIE/INTRUSION, ni SERVICES). Relevé sous « BOITIER C »,</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Symbole « $ » dans un carré avec bulle 1 et E.A.R à (1003 ; 552). Note spécifique 1 : « Interrupteurs maîtres, à</t>
+          <t>famille `autre`, matériel suffixé (hors legende). À identifier (contact de porte ? bouton de sortie ?).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>relocaliser. Tout l'éclairage de la zone principale du hall est commandé à partir de ce panneau. Système de</t>
+          <t>## R-007 — Interrupteurs maîtres (note spécifique 1)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>dénomination : Ma (Main a). » Relevé 1 repère `RELOCALISER`, hors légende. Les suffixes (Ma)/(Mf) des encastrés</t>
+          <t>Symbole « $ » dans un carré avec bulle 1 et E.A.R à (1003 ; 552). Note spécifique 1 : « Interrupteurs maîtres, à</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>renvoient à ce système.</t>
+          <t>relocaliser. Tout l'éclairage de la zone principale du hall est commandé à partir de ce panneau. Système de</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>## R-008 — Rails d'éclairage : quantité = 2 rails, têtes en désignation</t>
+          <t>dénomination : Ma (Main a). » Relevé 1 repère `RELOCALISER`, hors légende. Les suffixes (Ma)/(Mf) des encastrés</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Deux rails courbes (P-2 39 : 5 têtes, ~125 pt ≈ 4,4 m à 1:100 ; P-2 41 : 3 têtes, ~55 pt ≈ 1,9 m), tous deux</t>
+          <t>renvoient à ce système.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>E.A.E. Longueur estimée depuis l'échelle 1:100 du cartouche (1 pt = 0,0353 m) : **à métrer** avant chiffrage.</t>
+          <t>## R-008 — Rails d'éclairage : quantité = 2 rails, têtes en désignation</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Boîte de jonction (carré X) en tête de chaque rail relevée séparément (S01).</t>
+          <t>Deux rails courbes (P-2 39 : 5 têtes, ~125 pt ≈ 4,4 m à 1:100 ; P-2 41 : 3 têtes, ~55 pt ≈ 1,9 m), tous deux</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>## R-009 — Accumulateur (476 ; 610) sans étiquette</t>
+          <t>E.A.E. Longueur estimée depuis l'échelle 1:100 du cartouche (1 pt = 0,0353 m) : **à métrer** avant chiffrage.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rectangle « + − » avec un petit cercle accolé, à l'entrée du bureau 110.5. Relevé sous U04 « ACCUMULATEUR »,</t>
+          <t>Boîte de jonction (carré X) en tête de chaque rail relevée séparément (S01).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>`CONSERVER` (aucune mention E.A.E lue). Le petit cercle pourrait indiquer un phare : à confirmer.</t>
+          <t>## R-009 — Accumulateur (476 ; 610) sans étiquette</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>## R-010 — Lignes de légende absentes</t>
+          <t>Rectangle « + − » avec un petit cercle accolé, à l'entrée du bureau 110.5. Relevé sous U04 « ACCUMULATEUR »,</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>L02 (rectangle sans description), L03 réglette 4', L08 gradateur, L09 mural, L10/L11 réglettes murales, L13</t>
+          <t>`CONSERVER` (aucune mention E.A.E lue). Le petit cercle pourrait indiquer un phare : à confirmer.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>(hachuré, sans description), L15 347 V, L17 daylight, A02, A05, A07, A08, A10-A13, U03, U05-U10 : cherchées sur toute</t>
+          <t>## R-010 — Lignes de légende absentes</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>la zone blanche, aucune occurrence. Les sections SERVICES, DISTRIBUTION, CHAUFFAGE, FORCE MOTRICE de E-001 ne</t>
+          <t>L02 (rectangle sans description), L03 réglette 4', L08 gradateur, L09 mural, L10/L11 réglettes murales, L13</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>s'appliquent pas à une feuille d'éclairage/alarme (seule S01 boîte de jonction y figure).</t>
+          <t>(hachuré, sans description), L15 347 V, L17 daylight, A02, A05, A07, A08, A10-A13, U03, U05-U10 : cherchées sur toute</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>## R-011 — Limites du relevé</t>
+          <t>la zone blanche, aucune occurrence. Les sections SERVICES, DISTRIBUTION, CHAUFFAGE, FORCE MOTRICE de E-001 ne</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>- Entrée raster (PNG), pas le PDF vectoriel : `traits.py` inutilisable, coordonnées lues sur les règles des</t>
+          <t>s'appliquent pas à une feuille d'éclairage/alarme (seule S01 boîte de jonction y figure).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  zooms (précision ≈ ±1 pt) et par centroïde raster pour les appariements.</t>
+          <t>## R-012 — Vérification indépendante (12:30)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>- Aucun devis ni addenda fourni : colonne `modele` = EXISTANT CONSERVE - MODELE NON INDIQUE.</t>
+          <t>Un second agent, sans accès aux CSV ni au journal, a compté la feuille à l'aveugle (16 vignettes + légende) puis audité le</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>- Aucune référence d'estimateur : critère d'acceptation à l'étape 1 (identification à l'aveugle),</t>
+          <t>rendu : **0 écart de quantité** famille par famille (121/121, portées comprises), 0 omission, 0 faux positif ; 4 familles</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  **vérification incomplète**.</t>
+          <t>(R-004, corrigé), 3 décalages sûrs + 2 probables (I05-01, I05-02, M08-01, M10-01, M13-02 : corrigés par lecture au ×12/×14),</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
+        <is>
+          <t>4 doutes conservés (M01-01 accumulateur seul ou « 1 phare » ; M12-01 enseigne au bord de la zone grise ; M05-01/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>cercles sans étiquette, architecture probable). Rapport : `RAPPORT-VERIFICATEUR.md`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>## R-011 — Limites du relevé</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>- Entrée raster (PNG), pas le PDF vectoriel : `traits.py` inutilisable, coordonnées lues sur les règles des</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  zooms (précision ≈ ±1 pt) et par centroïde raster pour les appariements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>- Aucun devis ni addenda fourni : colonne `modele` = EXISTANT CONSERVE - MODELE NON INDIQUE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>- Aucune référence d'estimateur : critère d'acceptation à l'étape 1 (identification à l'aveugle),</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  **vérification incomplète**.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>- Modèle exécutant ce relevé : Claude Fable 5.1 (session interactive, route « session = agent » de CLAUDE.md).</t>
         </is>

</xml_diff>